<commit_message>
feat: add price extraction scripts and update 7 product prices from catalog data
</commit_message>
<xml_diff>
--- a/oil/Tomobile_Inventory_Complete.xlsx
+++ b/oil/Tomobile_Inventory_Complete.xlsx
@@ -683,19 +683,19 @@
         <v>81</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>61</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>59</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6">
@@ -708,19 +708,19 @@
         <v>78</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>13</v>
+        <v>78</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>13</v>
+        <v>78</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -733,19 +733,19 @@
         <v>32</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>13</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
@@ -783,19 +783,19 @@
         <v>201</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>97</v>
+        <v>198</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>97</v>
+        <v>201</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>97</v>
+        <v>146</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>97</v>
+        <v>178</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>95</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -822,7 +822,7 @@
     <row r="14">
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>• All data compiled: 2026-08-14 03:45</t>
+          <t>• All data compiled: 2026-08-14 16:34</t>
         </is>
       </c>
     </row>
@@ -4360,11 +4360,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E66" s="19" t="inlineStr"/>
-      <c r="F66" s="19" t="inlineStr"/>
+      <c r="E66" s="19" t="inlineStr">
+        <is>
+          <t>11.90</t>
+        </is>
+      </c>
+      <c r="F66" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G66" s="19" t="inlineStr"/>
       <c r="H66" s="19" t="inlineStr"/>
-      <c r="I66" s="19" t="inlineStr"/>
+      <c r="I66" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/1f23d0e5-7f95-44e4-bc3f-1bdc0201ff00/w=1040</t>
+        </is>
+      </c>
       <c r="J66" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/liquides-de-frein/mannol-liquide-de-frein-dot-4/</t>
@@ -4387,11 +4399,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E67" s="16" t="inlineStr"/>
-      <c r="F67" s="16" t="inlineStr"/>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>47.90</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G67" s="16" t="inlineStr"/>
       <c r="H67" s="16" t="inlineStr"/>
-      <c r="I67" s="16" t="inlineStr"/>
+      <c r="I67" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/64a6de30-8619-4762-c5ff-f9092271c800/w=1200</t>
+        </is>
+      </c>
       <c r="J67" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/mannol-aqua-jet-4-temps-10w-40/</t>
@@ -4414,11 +4438,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E68" s="19" t="inlineStr"/>
-      <c r="F68" s="19" t="inlineStr"/>
+      <c r="E68" s="19" t="inlineStr">
+        <is>
+          <t>29.90</t>
+        </is>
+      </c>
+      <c r="F68" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G68" s="19" t="inlineStr"/>
       <c r="H68" s="19" t="inlineStr"/>
-      <c r="I68" s="19" t="inlineStr"/>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/3031f4f2-fcda-4a6d-0e82-c03d99405a00/w=1040</t>
+        </is>
+      </c>
       <c r="J68" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/mannol-huile-hors-board-1l/</t>
@@ -4441,11 +4477,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E69" s="16" t="inlineStr"/>
-      <c r="F69" s="16" t="inlineStr"/>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>59.90</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G69" s="16" t="inlineStr"/>
       <c r="H69" s="16" t="inlineStr"/>
-      <c r="I69" s="16" t="inlineStr"/>
+      <c r="I69" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/8f7dda28-f66d-4354-17e3-002d14535700/w=1040</t>
+        </is>
+      </c>
       <c r="J69" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/mannol-huile-marine-outboard-2t-4l/</t>
@@ -4468,11 +4516,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E70" s="19" t="inlineStr"/>
-      <c r="F70" s="19" t="inlineStr"/>
+      <c r="E70" s="19" t="inlineStr">
+        <is>
+          <t>44.90</t>
+        </is>
+      </c>
+      <c r="F70" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G70" s="19" t="inlineStr"/>
       <c r="H70" s="19" t="inlineStr"/>
-      <c r="I70" s="19" t="inlineStr"/>
+      <c r="I70" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/dca03e4a-03cb-458a-37ea-e37497142a00/w=1040</t>
+        </is>
+      </c>
       <c r="J70" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/mannol-outboard-universel-1l/</t>
@@ -4495,11 +4555,27 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E71" s="16" t="inlineStr"/>
-      <c r="F71" s="16" t="inlineStr"/>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>24.90</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G71" s="16" t="inlineStr"/>
-      <c r="H71" s="16" t="inlineStr"/>
-      <c r="I71" s="16" t="inlineStr"/>
+      <c r="H71" s="16" t="inlineStr">
+        <is>
+          <t>MANNOL huile moto 4 temps 20W-50 1L</t>
+        </is>
+      </c>
+      <c r="I71" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/1b4ec910-7cd7-4a69-921a-b9b137981600/w=1040</t>
+        </is>
+      </c>
       <c r="J71" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/mannol-huile-moteur-motorbike/mannol-huile-4-temps-power-plus-15w-50/</t>
@@ -4522,11 +4598,27 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E72" s="19" t="inlineStr"/>
-      <c r="F72" s="19" t="inlineStr"/>
+      <c r="E72" s="19" t="inlineStr">
+        <is>
+          <t>1,084.90</t>
+        </is>
+      </c>
+      <c r="F72" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G72" s="19" t="inlineStr"/>
-      <c r="H72" s="19" t="inlineStr"/>
-      <c r="I72" s="19" t="inlineStr"/>
+      <c r="H72" s="19" t="inlineStr">
+        <is>
+          <t>💡 12 LED haute performance, portée 300 mètres.</t>
+        </is>
+      </c>
+      <c r="I72" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/32b2c809-6ca4-4bd6-52a1-62c222e1ad00/w=1040</t>
+        </is>
+      </c>
       <c r="J72" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/mannol-huile-moteur-motorbike/mannol-huile-moto-2-temps-plus-4-litres/</t>
@@ -4549,10 +4641,22 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E73" s="16" t="inlineStr"/>
-      <c r="F73" s="16" t="inlineStr"/>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>29.90</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G73" s="16" t="inlineStr"/>
-      <c r="H73" s="16" t="inlineStr"/>
+      <c r="H73" s="16" t="inlineStr">
+        <is>
+          <t>💡 Blanc bleuté intense jusqu’à 4200K aspect xénon premium</t>
+        </is>
+      </c>
       <c r="I73" s="16" t="inlineStr"/>
       <c r="J73" s="17" t="inlineStr">
         <is>
@@ -4576,11 +4680,27 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E74" s="19" t="inlineStr"/>
-      <c r="F74" s="19" t="inlineStr"/>
+      <c r="E74" s="19" t="inlineStr">
+        <is>
+          <t>9.90</t>
+        </is>
+      </c>
+      <c r="F74" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G74" s="19" t="inlineStr"/>
-      <c r="H74" s="19" t="inlineStr"/>
-      <c r="I74" s="19" t="inlineStr"/>
+      <c r="H74" s="19" t="inlineStr">
+        <is>
+          <t>💡 Ampoule halogène H7 55W 12V — culot PX26d, catégorie ECE H7</t>
+        </is>
+      </c>
+      <c r="I74" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/18597199-af9e-4a95-d482-37a6074dee00/w=1040</t>
+        </is>
+      </c>
       <c r="J74" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/mannol-huile-moteur-motorbike/mannol-huile-synthetique-4-temps-5w40/</t>
@@ -4603,11 +4723,27 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E75" s="16" t="inlineStr"/>
-      <c r="F75" s="16" t="inlineStr"/>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>42.90</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G75" s="16" t="inlineStr"/>
-      <c r="H75" s="16" t="inlineStr"/>
-      <c r="I75" s="16" t="inlineStr"/>
+      <c r="H75" s="16" t="inlineStr">
+        <is>
+          <t>💡 100% plus de lumière que la norme légale minimum</t>
+        </is>
+      </c>
+      <c r="I75" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/110d4ce0-a940-4e5a-bfba-92208e731f00/w=1040</t>
+        </is>
+      </c>
       <c r="J75" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/mannol-huile-moteur-motorbike/mannol-huile-4-temps-10w30-1l/</t>
@@ -4630,11 +4766,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E76" s="19" t="inlineStr"/>
-      <c r="F76" s="19" t="inlineStr"/>
+      <c r="E76" s="19" t="inlineStr">
+        <is>
+          <t>24.90</t>
+        </is>
+      </c>
+      <c r="F76" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G76" s="19" t="inlineStr"/>
       <c r="H76" s="19" t="inlineStr"/>
-      <c r="I76" s="19" t="inlineStr"/>
+      <c r="I76" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/6d4c28f8-91c2-4371-0f57-633052537700/w=1040</t>
+        </is>
+      </c>
       <c r="J76" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/mannol-huile-moteur-motorbike/mannol-huile-2-temps-1l/</t>
@@ -4657,11 +4805,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E77" s="16" t="inlineStr"/>
-      <c r="F77" s="16" t="inlineStr"/>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>26.90</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G77" s="16" t="inlineStr"/>
       <c r="H77" s="16" t="inlineStr"/>
-      <c r="I77" s="16" t="inlineStr"/>
+      <c r="I77" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/2628c649-af35-4e8f-bbf8-77e3da546500/w=1040</t>
+        </is>
+      </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/mannol-huile-moteur-motorbike/mannol-4-temps-plus-10w-40-1l/</t>
@@ -4684,11 +4844,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E78" s="19" t="inlineStr"/>
-      <c r="F78" s="19" t="inlineStr"/>
+      <c r="E78" s="19" t="inlineStr">
+        <is>
+          <t>36.90</t>
+        </is>
+      </c>
+      <c r="F78" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G78" s="19" t="inlineStr"/>
       <c r="H78" s="19" t="inlineStr"/>
-      <c r="I78" s="19" t="inlineStr"/>
+      <c r="I78" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/4b19bf50-d8b0-4259-c4ae-d61a28a67a00/w=1040</t>
+        </is>
+      </c>
       <c r="J78" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huiles-pour-fourche/mannol-huile-de-fourche-10w-1l/</t>
@@ -4711,11 +4883,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E79" s="16" t="inlineStr"/>
-      <c r="F79" s="16" t="inlineStr"/>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>49.90</t>
+        </is>
+      </c>
+      <c r="F79" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G79" s="16" t="inlineStr"/>
       <c r="H79" s="16" t="inlineStr"/>
-      <c r="I79" s="16" t="inlineStr"/>
+      <c r="I79" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/09133af8-495f-4578-4787-c9a0bdb11b00/w=1080</t>
+        </is>
+      </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/mannol-pack-entretien-chaine/</t>
@@ -4738,11 +4922,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E80" s="19" t="inlineStr"/>
-      <c r="F80" s="19" t="inlineStr"/>
+      <c r="E80" s="19" t="inlineStr">
+        <is>
+          <t>20.90</t>
+        </is>
+      </c>
+      <c r="F80" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G80" s="19" t="inlineStr"/>
       <c r="H80" s="19" t="inlineStr"/>
-      <c r="I80" s="19" t="inlineStr"/>
+      <c r="I80" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/f1962794-b383-464a-b17c-26d8ff869a00/w=1200</t>
+        </is>
+      </c>
       <c r="J80" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/mannol-lubrifiant-m-40-400ml/</t>
@@ -4765,11 +4961,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E81" s="16" t="inlineStr"/>
-      <c r="F81" s="16" t="inlineStr"/>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G81" s="16" t="inlineStr"/>
       <c r="H81" s="16" t="inlineStr"/>
-      <c r="I81" s="16" t="inlineStr"/>
+      <c r="I81" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/6f017b18-8c8a-41a8-5e4a-9595bce3c900/w=400</t>
+        </is>
+      </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/chaine-motorbike/mannol-nettoyant-chaine-400-ml/</t>
@@ -4792,11 +5000,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E82" s="19" t="inlineStr"/>
-      <c r="F82" s="19" t="inlineStr"/>
+      <c r="E82" s="19" t="inlineStr">
+        <is>
+          <t>19.90</t>
+        </is>
+      </c>
+      <c r="F82" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G82" s="19" t="inlineStr"/>
       <c r="H82" s="19" t="inlineStr"/>
-      <c r="I82" s="19" t="inlineStr"/>
+      <c r="I82" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/36c7218f-53c4-4e6b-b93f-eaf6d819be00/w=1040</t>
+        </is>
+      </c>
       <c r="J82" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/mannol-liquide-de-refroidissement-moto-pro-cool-1l/</t>
@@ -4819,11 +5039,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E83" s="16" t="inlineStr"/>
-      <c r="F83" s="16" t="inlineStr"/>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>15.90</t>
+        </is>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G83" s="16" t="inlineStr"/>
       <c r="H83" s="16" t="inlineStr"/>
-      <c r="I83" s="16" t="inlineStr"/>
+      <c r="I83" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/e902108d-f034-441c-1bbe-d3aae1fb6900/w=2362</t>
+        </is>
+      </c>
       <c r="J83" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-essence/mannol-nettoyant-injecteurs-essence-400ml/</t>
@@ -4846,11 +5078,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E84" s="19" t="inlineStr"/>
-      <c r="F84" s="19" t="inlineStr"/>
+      <c r="E84" s="19" t="inlineStr">
+        <is>
+          <t>17.90</t>
+        </is>
+      </c>
+      <c r="F84" s="19" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G84" s="19" t="inlineStr"/>
       <c r="H84" s="19" t="inlineStr"/>
-      <c r="I84" s="19" t="inlineStr"/>
+      <c r="I84" s="20" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/7f211033-cf00-4e9f-7dec-63055ecdb900/w=400</t>
+        </is>
+      </c>
       <c r="J84" s="20" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/nettoyant-injection/mannol-nettoyant-injecteurs-diesel-250ml/</t>
@@ -4873,11 +5117,23 @@
           <t>Mannol</t>
         </is>
       </c>
-      <c r="E85" s="16" t="inlineStr"/>
-      <c r="F85" s="16" t="inlineStr"/>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>19.90</t>
+        </is>
+      </c>
+      <c r="F85" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G85" s="16" t="inlineStr"/>
       <c r="H85" s="16" t="inlineStr"/>
-      <c r="I85" s="16" t="inlineStr"/>
+      <c r="I85" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/7019a63f-0716-4157-6ffb-c7f8742c8600/w=680</t>
+        </is>
+      </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/gamme-atelier/lmannol-lithium-spray-400ml/</t>
@@ -5013,26 +5269,45 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId161"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5800,17 +6075,33 @@
           <t>liqui-moly-additif-diesel-5-en-1-pro-line</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr"/>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>LM21535</t>
+        </is>
+      </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr"/>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F18" s="22" t="inlineStr"/>
       <c r="G18" s="22" t="inlineStr"/>
-      <c r="H18" s="22" t="inlineStr"/>
-      <c r="I18" s="22" t="inlineStr"/>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a539fb5d-8f12-4235-f875-0f6299266700/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-diesel/liqui-moly-additif-diesel-5-en-1-pro-line/</t>
@@ -5827,17 +6118,33 @@
           <t>liqui-moly-super-additif-diesel-250ml</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr"/>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>LM8366</t>
+        </is>
+      </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr"/>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="16" t="inlineStr"/>
-      <c r="H19" s="16" t="inlineStr"/>
-      <c r="I19" s="16" t="inlineStr"/>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/fc3c25d7-1c2c-4e44-1f58-d1285062f300/w=1000,h=1000,fit=crop</t>
+        </is>
+      </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-diesel/liqui-moly-super-additif-diesel-250ml/</t>
@@ -5854,17 +6161,33 @@
           <t>liqui-moly-additif-common-rail-250ml</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr"/>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>LM8372</t>
+        </is>
+      </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E20" s="22" t="inlineStr"/>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F20" s="22" t="inlineStr"/>
       <c r="G20" s="22" t="inlineStr"/>
-      <c r="H20" s="22" t="inlineStr"/>
-      <c r="I20" s="22" t="inlineStr"/>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I20" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a38d88e6-f627-4de4-5349-e32d5b81e800/w=444,h=444,fit=crop</t>
+        </is>
+      </c>
       <c r="J20" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-huile/liqui-moly-additif-common-rail-250ml/</t>
@@ -5881,17 +6204,33 @@
           <t>liqui-moly-createc</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr"/>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>LM3721</t>
+        </is>
+      </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr"/>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F21" s="16" t="inlineStr"/>
       <c r="G21" s="16" t="inlineStr"/>
-      <c r="H21" s="16" t="inlineStr"/>
-      <c r="I21" s="16" t="inlineStr"/>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/486fa1f3-c49d-4707-775e-1ceaa9f10f00/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-huile/liqui-moly-createc/</t>
@@ -5908,17 +6247,33 @@
           <t>liqui-moly-rincage-boue-dhuile</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr"/>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>LM5200</t>
+        </is>
+      </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr"/>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F22" s="22" t="inlineStr"/>
       <c r="G22" s="22" t="inlineStr"/>
-      <c r="H22" s="22" t="inlineStr"/>
-      <c r="I22" s="22" t="inlineStr"/>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/7ddd8552-bd07-4a06-f814-e12a4b0a9200/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J22" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-huile/liqui-moly-rincage-boue-dhuile/</t>
@@ -5935,17 +6290,33 @@
           <t>liqui-moly-rincage-moteur-300ml</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr"/>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>LM8993</t>
+        </is>
+      </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr"/>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F23" s="16" t="inlineStr"/>
       <c r="G23" s="16" t="inlineStr"/>
-      <c r="H23" s="16" t="inlineStr"/>
-      <c r="I23" s="16" t="inlineStr"/>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/57dcf71c-291f-4db8-791e-5bc2bad62800/w=800,h=1080</t>
+        </is>
+      </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-huile/liqui-moly-rincage-moteur-300ml/</t>
@@ -5962,17 +6333,33 @@
           <t>liqui-moly-mousse-dentretien-textile</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr"/>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>LM1539</t>
+        </is>
+      </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr"/>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F24" s="22" t="inlineStr"/>
       <c r="G24" s="22" t="inlineStr"/>
-      <c r="H24" s="22" t="inlineStr"/>
-      <c r="I24" s="22" t="inlineStr"/>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I24" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/80b3bc0b-59f3-45ac-5bb4-96eb85966f00/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J24" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/detailing/interieure-produits-de-nettoyage/cuir-textile/liqui-moly-mousse-dentretien-textile/</t>
@@ -5989,17 +6376,33 @@
           <t>liqui-moly-motorbike-4t-bike-additive</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr"/>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>LM1581</t>
+        </is>
+      </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr"/>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="16" t="inlineStr"/>
-      <c r="H25" s="16" t="inlineStr"/>
-      <c r="I25" s="16" t="inlineStr"/>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/f5fc4600-c8ae-4026-7734-8ab1668a4800/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/additifs-moto/additif-essence/liqui-moly-motorbike-4t-bike-additive/</t>
@@ -6016,17 +6419,33 @@
           <t>liqui-moly-motorbike-additif-huile-2t-et-4t-125ml</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr"/>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>LM1580</t>
+        </is>
+      </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr"/>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F26" s="22" t="inlineStr"/>
       <c r="G26" s="22" t="inlineStr"/>
-      <c r="H26" s="22" t="inlineStr"/>
-      <c r="I26" s="22" t="inlineStr"/>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I26" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/4cb56dde-9ab7-43a6-2ce7-6d9fdaa81400/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/additifs-moto/additif-huile/liqui-moly-motorbike-additif-huile-2t-et-4t-125ml/</t>
@@ -6043,17 +6462,37 @@
           <t>liqui-moly-motorbike-mos2-shooter</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr"/>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>LM3444</t>
+        </is>
+      </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr"/>
-      <c r="F27" s="16" t="inlineStr"/>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
       <c r="G27" s="16" t="inlineStr"/>
-      <c r="H27" s="16" t="inlineStr"/>
-      <c r="I27" s="16" t="inlineStr"/>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/58eb99d2-6612-4ea7-5667-065c3f45a100/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/additifs-moto/additif-huile/liqui-moly-motorbike-mos2-shooter/</t>
@@ -6070,17 +6509,33 @@
           <t>liqui-moly-molygen-4t-10w-40-scooter-1l</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr"/>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>LM21719</t>
+        </is>
+      </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr"/>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F28" s="22" t="inlineStr"/>
       <c r="G28" s="22" t="inlineStr"/>
-      <c r="H28" s="22" t="inlineStr"/>
-      <c r="I28" s="22" t="inlineStr"/>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I28" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/17e4e639-711f-4f91-217c-071d74f29e00/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/liqui-moly-huile-moteur-motorbike/liqui-moly-molygen-4t-10w-40-scooter-1l/</t>
@@ -6097,17 +6552,33 @@
           <t>liqui-moly-motorbike-4t-synth-10w-40-scooter-mb</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr"/>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>LM20832</t>
+        </is>
+      </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr"/>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F29" s="16" t="inlineStr"/>
       <c r="G29" s="16" t="inlineStr"/>
-      <c r="H29" s="16" t="inlineStr"/>
-      <c r="I29" s="16" t="inlineStr"/>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/b1a65fc2-e7da-4b0e-1e3b-9d7a58026d00/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/liqui-moly-huile-moteur-motorbike/liqui-moly-motorbike-4t-synth-10w-40-scooter-mb/</t>
@@ -6124,17 +6595,33 @@
           <t>liqui-moly-motorbike-4t-synth-street-race-1l</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr"/>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>LM1505</t>
+        </is>
+      </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr"/>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F30" s="22" t="inlineStr"/>
       <c r="G30" s="22" t="inlineStr"/>
-      <c r="H30" s="22" t="inlineStr"/>
-      <c r="I30" s="22" t="inlineStr"/>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I30" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/4eb9cb6c-53f2-49c9-a3ab-cdd65f387d00/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/liqui-moly-huile-moteur-motorbike/liqui-moly-motorbike-4t-synth-street-race-1l/</t>
@@ -6151,17 +6638,33 @@
           <t>liqui-moly-huile-de-boite-moto-75w-140-gl5</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr"/>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>LM3072</t>
+        </is>
+      </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr"/>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="16" t="inlineStr"/>
-      <c r="H31" s="16" t="inlineStr"/>
-      <c r="I31" s="16" t="inlineStr"/>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/1750d0d3-53ca-43e0-48c6-d44f87173a00/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-transmission/liqui-moly-huile-de-boite-moto-75w-140-gl5/</t>
@@ -6178,17 +6681,33 @@
           <t>liqui-moly-additif-anti-cristallisation-adblue-concentre</t>
         </is>
       </c>
-      <c r="C32" s="21" t="inlineStr"/>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>LM21799</t>
+        </is>
+      </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr"/>
+      <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F32" s="22" t="inlineStr"/>
       <c r="G32" s="22" t="inlineStr"/>
-      <c r="H32" s="22" t="inlineStr"/>
-      <c r="I32" s="22" t="inlineStr"/>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I32" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/70bb4a61-5ab5-4b9e-effc-25d8bfc52800/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-diesel/liqui-moly-additif-anti-cristallisation-adblue-concentre/</t>
@@ -6205,17 +6724,33 @@
           <t>liqui-moly-hybrid-additive-250ml</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr"/>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>lm1001</t>
+        </is>
+      </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr"/>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F33" s="16" t="inlineStr"/>
       <c r="G33" s="16" t="inlineStr"/>
-      <c r="H33" s="16" t="inlineStr"/>
-      <c r="I33" s="16" t="inlineStr"/>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/b07babf9-c39e-4e2a-b751-ed158e6d2600/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J33" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-essence/liqui-moly-hybrid-additive-250ml/</t>
@@ -6232,17 +6767,33 @@
           <t>liqui-moly-additif-essence-5-en-1-300ml</t>
         </is>
       </c>
-      <c r="C34" s="21" t="inlineStr"/>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>lm21536</t>
+        </is>
+      </c>
       <c r="D34" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr"/>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F34" s="22" t="inlineStr"/>
       <c r="G34" s="22" t="inlineStr"/>
-      <c r="H34" s="22" t="inlineStr"/>
-      <c r="I34" s="22" t="inlineStr"/>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I34" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/de63e429-6243-42ad-26d8-c157fd0c4400/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-essence/liqui-moly-additif-essence-5-en-1-300ml/</t>
@@ -6259,17 +6810,33 @@
           <t>liqui-moly-nettoyant-injection-directe-pro-line</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr"/>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>LM21281</t>
+        </is>
+      </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr"/>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F35" s="16" t="inlineStr"/>
       <c r="G35" s="16" t="inlineStr"/>
-      <c r="H35" s="16" t="inlineStr"/>
-      <c r="I35" s="16" t="inlineStr"/>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/f8ddc69a-ee4b-44cd-a3d2-95827ef53c00/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J35" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-essence/liqui-moly-nettoyant-injection-directe-pro-line/</t>
@@ -6286,17 +6853,33 @@
           <t>liqui-moly-motor-protect-500ml</t>
         </is>
       </c>
-      <c r="C36" s="21" t="inlineStr"/>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>LM1018</t>
+        </is>
+      </c>
       <c r="D36" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr"/>
+      <c r="E36" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F36" s="22" t="inlineStr"/>
       <c r="G36" s="22" t="inlineStr"/>
-      <c r="H36" s="22" t="inlineStr"/>
-      <c r="I36" s="22" t="inlineStr"/>
+      <c r="H36" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I36" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/79093a76-f007-4ddc-4b53-da9f0d165000/w=320,h=361</t>
+        </is>
+      </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-huile/liqui-moly-motor-protect-500ml/</t>
@@ -6313,17 +6896,33 @@
           <t>liqui-moly-molygen-motor-protect-500ml</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr"/>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>LM1015</t>
+        </is>
+      </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E37" s="16" t="inlineStr"/>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="16" t="inlineStr"/>
-      <c r="H37" s="16" t="inlineStr"/>
-      <c r="I37" s="16" t="inlineStr"/>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I37" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/3369cb88-42fe-4cde-ef63-1527f1b9e500/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J37" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-huile/liqui-moly-molygen-motor-protect-500ml/</t>
@@ -6340,17 +6939,33 @@
           <t>liqui-moly-nettoyant-filtre-a-particule-fap-dpf</t>
         </is>
       </c>
-      <c r="C38" s="21" t="inlineStr"/>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>LM21942</t>
+        </is>
+      </c>
       <c r="D38" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr"/>
+      <c r="E38" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F38" s="22" t="inlineStr"/>
       <c r="G38" s="22" t="inlineStr"/>
-      <c r="H38" s="22" t="inlineStr"/>
-      <c r="I38" s="22" t="inlineStr"/>
+      <c r="H38" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I38" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/747ad558-69ba-41ba-df12-717dbfe6ec00/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-nettoyant-filtre-a-particule-fap-dpf/</t>
@@ -6367,17 +6982,37 @@
           <t>liqui-moly-protection-du-filte-a-particule-diesel-250ml</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr"/>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>LM5148</t>
+        </is>
+      </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E39" s="16" t="inlineStr"/>
-      <c r="F39" s="16" t="inlineStr"/>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
       <c r="G39" s="16" t="inlineStr"/>
-      <c r="H39" s="16" t="inlineStr"/>
-      <c r="I39" s="16" t="inlineStr"/>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I39" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/c1a231c5-a57a-4b88-8541-5a666681c800/w=450,h=450,fit=crop</t>
+        </is>
+      </c>
       <c r="J39" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-protection-du-filte-a-particule-diesel-250ml/</t>
@@ -6394,17 +7029,33 @@
           <t>liqui-moly-pack-nettoyage-catalyseur</t>
         </is>
       </c>
-      <c r="C40" s="21" t="inlineStr"/>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>Packcatalytic</t>
+        </is>
+      </c>
       <c r="D40" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr"/>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F40" s="22" t="inlineStr"/>
       <c r="G40" s="22" t="inlineStr"/>
-      <c r="H40" s="22" t="inlineStr"/>
-      <c r="I40" s="22" t="inlineStr"/>
+      <c r="H40" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/b2f8c6b9-10a2-4ac9-7afd-1967c5ac0a00/w=940,h=788</t>
+        </is>
+      </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-pack-nettoyage-catalyseur/</t>
@@ -6421,17 +7072,33 @@
           <t>liqui-moly-catalytic-system-clean-300ml</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr"/>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>LM7110</t>
+        </is>
+      </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E41" s="16" t="inlineStr"/>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F41" s="16" t="inlineStr"/>
       <c r="G41" s="16" t="inlineStr"/>
-      <c r="H41" s="16" t="inlineStr"/>
-      <c r="I41" s="16" t="inlineStr"/>
+      <c r="H41" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I41" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/05f601a4-f9c9-43a3-341b-8c1ec1369100/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J41" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-catalytic-system-clean-300ml/</t>
@@ -6448,17 +7115,33 @@
           <t>liqui-moly-nettoyant-pour-filtre-a-particules-fap-diesel-pro-line-1-litre</t>
         </is>
       </c>
-      <c r="C42" s="21" t="inlineStr"/>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>LM5169</t>
+        </is>
+      </c>
       <c r="D42" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr"/>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F42" s="22" t="inlineStr"/>
       <c r="G42" s="22" t="inlineStr"/>
-      <c r="H42" s="22" t="inlineStr"/>
-      <c r="I42" s="22" t="inlineStr"/>
+      <c r="H42" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I42" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/1cbd654c-932a-4889-f9c4-57261e83a200/w=800,h=800,fit=crop</t>
+        </is>
+      </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-nettoyant-pour-filtre-a-particules-fap-diesel-pro-line-1-litre/</t>
@@ -6475,17 +7158,33 @@
           <t>liqui-moly-catalytic-system-cleaner-300ml</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr"/>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>LM8931</t>
+        </is>
+      </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E43" s="16" t="inlineStr"/>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F43" s="16" t="inlineStr"/>
       <c r="G43" s="16" t="inlineStr"/>
-      <c r="H43" s="16" t="inlineStr"/>
-      <c r="I43" s="16" t="inlineStr"/>
+      <c r="H43" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I43" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/ee23b0d1-6967-4c2e-9309-3c8b556e1800/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J43" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-catalytic-system-cleaner-300ml/</t>
@@ -6502,17 +7201,37 @@
           <t>liqui-moly-liquide-de-rincage-pour-filtre-a-particules-fap-diesel-pro-line-500ml</t>
         </is>
       </c>
-      <c r="C44" s="21" t="inlineStr"/>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>LM5171</t>
+        </is>
+      </c>
       <c r="D44" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr"/>
-      <c r="F44" s="22" t="inlineStr"/>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
       <c r="G44" s="22" t="inlineStr"/>
-      <c r="H44" s="22" t="inlineStr"/>
-      <c r="I44" s="22" t="inlineStr"/>
+      <c r="H44" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I44" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/476325f8-61a1-463d-9b3d-f6d7af058b00/w=458,h=458,fit=crop</t>
+        </is>
+      </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/filtre-a-particule-fap/liqui-moly-liquide-de-rincage-pour-filtre-a-particules-fap-diesel-pro-line-500ml/</t>
@@ -6529,17 +7248,33 @@
           <t>liqui-moly-liquide-de-refroidissement-concentre-kfs-18</t>
         </is>
       </c>
-      <c r="C45" s="15" t="inlineStr"/>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>LM23152</t>
+        </is>
+      </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E45" s="16" t="inlineStr"/>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F45" s="16" t="inlineStr"/>
       <c r="G45" s="16" t="inlineStr"/>
-      <c r="H45" s="16" t="inlineStr"/>
-      <c r="I45" s="16" t="inlineStr"/>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/d9da5717-f84e-43ea-cc8b-1bd487471b00/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-radiateur/liqui-moly-liquide-de-refroidissement-concentre-kfs-18/</t>
@@ -6556,17 +7291,33 @@
           <t>liqui-moly-g11-pret-a-lemploi-50-50-5l</t>
         </is>
       </c>
-      <c r="C46" s="21" t="inlineStr"/>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>LM8809</t>
+        </is>
+      </c>
       <c r="D46" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr"/>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F46" s="22" t="inlineStr"/>
       <c r="G46" s="22" t="inlineStr"/>
-      <c r="H46" s="22" t="inlineStr"/>
-      <c r="I46" s="22" t="inlineStr"/>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I46" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/521fbe26-4ca7-45d5-eb31-e4f17aa89300/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-radiateur/liqui-moly-g11-pret-a-lemploi-50-50-5l/</t>
@@ -6583,17 +7334,33 @@
           <t>liqui-moly-shampoing-auto-avec-cire</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr"/>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>LM23007</t>
+        </is>
+      </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E47" s="16" t="inlineStr"/>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F47" s="16" t="inlineStr"/>
       <c r="G47" s="16" t="inlineStr"/>
-      <c r="H47" s="16" t="inlineStr"/>
-      <c r="I47" s="16" t="inlineStr"/>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I47" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a727d3c6-73bc-4e3e-e0bb-bf8ef0ee2d00/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J47" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/detailing/exterieur/shampoing/liqui-moly-shampoing-auto-avec-cire/</t>
@@ -6610,17 +7377,33 @@
           <t>liqui-moly-top-tec-atf-1800-r</t>
         </is>
       </c>
-      <c r="C48" s="21" t="inlineStr"/>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>LM20625</t>
+        </is>
+      </c>
       <c r="D48" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr"/>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F48" s="22" t="inlineStr"/>
       <c r="G48" s="22" t="inlineStr"/>
-      <c r="H48" s="22" t="inlineStr"/>
-      <c r="I48" s="22" t="inlineStr"/>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I48" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/c180451e-7722-4695-4d19-3d18a8be6c00/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/huiles-de-boite-pont-direction/liqui-moly-top-tec-atf-1800-r/</t>
@@ -6637,17 +7420,33 @@
           <t>liqui-moly-huile-pour-systeme-hydraulique-central-1l</t>
         </is>
       </c>
-      <c r="C49" s="15" t="inlineStr"/>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>LM9524</t>
+        </is>
+      </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E49" s="16" t="inlineStr"/>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F49" s="16" t="inlineStr"/>
       <c r="G49" s="16" t="inlineStr"/>
-      <c r="H49" s="16" t="inlineStr"/>
-      <c r="I49" s="16" t="inlineStr"/>
+      <c r="H49" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I49" s="17" t="inlineStr">
+        <is>
+          <t>https://tomobile.store/wp-content/uploads/2025/11/661fc4bed9bb1708fe8379cc407761845ede34d6_1127_Zentralhydraulik__l_1l_745c.png</t>
+        </is>
+      </c>
       <c r="J49" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/huiles-de-boite-pont-direction/liqui-moly-huile-pour-systeme-hydraulique-central-1l/</t>
@@ -6664,17 +7463,33 @@
           <t>liqui-moly-liquide-de-frein-dot-3-500ml</t>
         </is>
       </c>
-      <c r="C50" s="21" t="inlineStr"/>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>LM3089</t>
+        </is>
+      </c>
       <c r="D50" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr"/>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F50" s="22" t="inlineStr"/>
       <c r="G50" s="22" t="inlineStr"/>
-      <c r="H50" s="22" t="inlineStr"/>
-      <c r="I50" s="22" t="inlineStr"/>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I50" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/b9003619-4cdf-4f4e-12d3-7ae9d5fc9300/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/liquides-de-frein/liqui-moly-liquide-de-frein-dot-3-500ml/</t>
@@ -6691,17 +7506,33 @@
           <t>liqui-moly-liquide-de-frein-dot-5-1-250ml</t>
         </is>
       </c>
-      <c r="C51" s="15" t="inlineStr"/>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>LM3092</t>
+        </is>
+      </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E51" s="16" t="inlineStr"/>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F51" s="16" t="inlineStr"/>
       <c r="G51" s="16" t="inlineStr"/>
-      <c r="H51" s="16" t="inlineStr"/>
-      <c r="I51" s="16" t="inlineStr"/>
+      <c r="H51" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/cc93dbc4-f941-4c85-fa26-041ba5bf8000/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J51" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/liquides-de-frein/liqui-moly-liquide-de-frein-dot-5-1-250ml/</t>
@@ -6718,17 +7549,33 @@
           <t>liqui-moly-liquide-de-frein-dot-4-250ml</t>
         </is>
       </c>
-      <c r="C52" s="21" t="inlineStr"/>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>LM3093</t>
+        </is>
+      </c>
       <c r="D52" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr"/>
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F52" s="22" t="inlineStr"/>
       <c r="G52" s="22" t="inlineStr"/>
-      <c r="H52" s="22" t="inlineStr"/>
-      <c r="I52" s="22" t="inlineStr"/>
+      <c r="H52" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I52" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/295b71ce-ce3d-4b9f-af7a-a5a1ec3bb100/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/liquides-de-frein/liqui-moly-liquide-de-frein-dot-4-250ml/</t>
@@ -6745,17 +7592,33 @@
           <t>liqui-moly-huile-marine-4t-10w-30</t>
         </is>
       </c>
-      <c r="C53" s="15" t="inlineStr"/>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>marine10w304t</t>
+        </is>
+      </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E53" s="16" t="inlineStr"/>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F53" s="16" t="inlineStr"/>
       <c r="G53" s="16" t="inlineStr"/>
-      <c r="H53" s="16" t="inlineStr"/>
-      <c r="I53" s="16" t="inlineStr"/>
+      <c r="H53" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I53" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/c229b80f-cfbb-4009-7235-da10d8a69000/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J53" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/liqui-moly-huile-marine-4t-10w-30/</t>
@@ -6772,17 +7635,33 @@
           <t>liqui-moly-huile-marine-4t-25w40-1l</t>
         </is>
       </c>
-      <c r="C54" s="21" t="inlineStr"/>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>LM25026</t>
+        </is>
+      </c>
       <c r="D54" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr"/>
+      <c r="E54" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F54" s="22" t="inlineStr"/>
       <c r="G54" s="22" t="inlineStr"/>
-      <c r="H54" s="22" t="inlineStr"/>
-      <c r="I54" s="22" t="inlineStr"/>
+      <c r="H54" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I54" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/12ec5836-f057-4424-e6b6-82311e821100/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J54" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/liqui-moly-huile-marine-4t-25w40-1l/</t>
@@ -6799,17 +7678,33 @@
           <t>liqui-moly-marine-2t-dfi-motor-oil-5l</t>
         </is>
       </c>
-      <c r="C55" s="15" t="inlineStr"/>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>LM25063</t>
+        </is>
+      </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E55" s="16" t="inlineStr"/>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F55" s="16" t="inlineStr"/>
       <c r="G55" s="16" t="inlineStr"/>
-      <c r="H55" s="16" t="inlineStr"/>
-      <c r="I55" s="16" t="inlineStr"/>
+      <c r="H55" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I55" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/34339698-c341-40ea-6cfd-a49d6ffd4700/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J55" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/liqui-moly-marine-2t-dfi-motor-oil-5l/</t>
@@ -6826,17 +7721,33 @@
           <t>liqui-moly-huile-marine-4t-10w-40</t>
         </is>
       </c>
-      <c r="C56" s="21" t="inlineStr"/>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>Marine10w40-4T</t>
+        </is>
+      </c>
       <c r="D56" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr"/>
+      <c r="E56" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F56" s="22" t="inlineStr"/>
       <c r="G56" s="22" t="inlineStr"/>
-      <c r="H56" s="22" t="inlineStr"/>
-      <c r="I56" s="22" t="inlineStr"/>
+      <c r="H56" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I56" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/ae2d2223-66be-4e0d-461d-3eb497f2de00/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J56" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/huiles-marine/liqui-moly-huile-marine-4t-10w-40/</t>
@@ -6853,17 +7764,33 @@
           <t>liqui-moly-marine-multispray</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr"/>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>LM25051</t>
+        </is>
+      </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E57" s="16" t="inlineStr"/>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F57" s="16" t="inlineStr"/>
       <c r="G57" s="16" t="inlineStr"/>
-      <c r="H57" s="16" t="inlineStr"/>
-      <c r="I57" s="16" t="inlineStr"/>
+      <c r="H57" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I57" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/1d4e3cc3-45c3-43a3-0e2c-71fcafeb6700/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J57" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/entretien-bateau/liqui-moly-marine-multispray/</t>
@@ -6880,17 +7807,33 @@
           <t>liqui-moly-marine-protection-gazole-500ml</t>
         </is>
       </c>
-      <c r="C58" s="21" t="inlineStr"/>
+      <c r="C58" s="21" t="inlineStr">
+        <is>
+          <t>LM25000</t>
+        </is>
+      </c>
       <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr"/>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F58" s="22" t="inlineStr"/>
       <c r="G58" s="22" t="inlineStr"/>
-      <c r="H58" s="22" t="inlineStr"/>
-      <c r="I58" s="22" t="inlineStr"/>
+      <c r="H58" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I58" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/ed871f45-1d9e-45bf-5129-a6fc1b982400/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J58" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/entretien-bateau/liqui-moly-marine-protection-gazole-500ml/</t>
@@ -6907,17 +7850,33 @@
           <t>liqui-moly-marine-super-diesel-additiv</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr"/>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>LM25005</t>
+        </is>
+      </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E59" s="16" t="inlineStr"/>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F59" s="16" t="inlineStr"/>
       <c r="G59" s="16" t="inlineStr"/>
-      <c r="H59" s="16" t="inlineStr"/>
-      <c r="I59" s="16" t="inlineStr"/>
+      <c r="H59" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I59" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/dcc998c4-0f2d-47bd-2837-17b9a7d8d200/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J59" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/entretien-bateau/liqui-moly-marine-super-diesel-additiv/</t>
@@ -6934,17 +7893,33 @@
           <t>liqui-moly-additif-diesel-anti-bacterien-1l</t>
         </is>
       </c>
-      <c r="C60" s="21" t="inlineStr"/>
+      <c r="C60" s="21" t="inlineStr">
+        <is>
+          <t>LM21317</t>
+        </is>
+      </c>
       <c r="D60" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E60" s="22" t="inlineStr"/>
+      <c r="E60" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F60" s="22" t="inlineStr"/>
       <c r="G60" s="22" t="inlineStr"/>
-      <c r="H60" s="22" t="inlineStr"/>
-      <c r="I60" s="22" t="inlineStr"/>
+      <c r="H60" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I60" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/ccb7ef8e-96c7-4b66-ba11-fb61b1cfd900/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J60" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/additifs-auto/additifs-diesel/liqui-moly-additif-diesel-anti-bacterien-1l/</t>
@@ -6961,17 +7936,33 @@
           <t>liqui-moly-entretien-circuits-dinjection-marine</t>
         </is>
       </c>
-      <c r="C61" s="15" t="inlineStr"/>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>LM25011</t>
+        </is>
+      </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E61" s="16" t="inlineStr"/>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F61" s="16" t="inlineStr"/>
       <c r="G61" s="16" t="inlineStr"/>
-      <c r="H61" s="16" t="inlineStr"/>
-      <c r="I61" s="16" t="inlineStr"/>
+      <c r="H61" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I61" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a4a7a10a-d755-45e0-5240-2c9b7e40dc00/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J61" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/entretien-bateau/liqui-moly-entretien-circuits-dinjection-marine/</t>
@@ -6988,17 +7979,33 @@
           <t>liqui-moly-protection-interieure-du-moteur-marine</t>
         </is>
       </c>
-      <c r="C62" s="21" t="inlineStr"/>
+      <c r="C62" s="21" t="inlineStr">
+        <is>
+          <t>LM25032</t>
+        </is>
+      </c>
       <c r="D62" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E62" s="22" t="inlineStr"/>
+      <c r="E62" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F62" s="22" t="inlineStr"/>
       <c r="G62" s="22" t="inlineStr"/>
-      <c r="H62" s="22" t="inlineStr"/>
-      <c r="I62" s="22" t="inlineStr"/>
+      <c r="H62" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I62" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/b1732d98-b6ff-4f19-1696-e2679f54ab00/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J62" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/entretien-bateau/liqui-moly-protection-interieure-du-moteur-marine/</t>
@@ -7015,17 +8022,33 @@
           <t>liqui-moly-marine-stabilisateur-dessence</t>
         </is>
       </c>
-      <c r="C63" s="15" t="inlineStr"/>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>LM25008</t>
+        </is>
+      </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E63" s="16" t="inlineStr"/>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F63" s="16" t="inlineStr"/>
       <c r="G63" s="16" t="inlineStr"/>
-      <c r="H63" s="16" t="inlineStr"/>
-      <c r="I63" s="16" t="inlineStr"/>
+      <c r="H63" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I63" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/38d55da0-c69f-4efe-a08c-64b76f3ed900/w=547,h=539</t>
+        </is>
+      </c>
       <c r="J63" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/marine/entretien-bateau/liqui-moly-marine-stabilisateur-dessence/</t>
@@ -7042,17 +8065,33 @@
           <t>liqui-moly-motorbike-4t-10w-30-street-1l</t>
         </is>
       </c>
-      <c r="C64" s="21" t="inlineStr"/>
+      <c r="C64" s="21" t="inlineStr">
+        <is>
+          <t>lm2526</t>
+        </is>
+      </c>
       <c r="D64" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E64" s="22" t="inlineStr"/>
+      <c r="E64" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F64" s="22" t="inlineStr"/>
       <c r="G64" s="22" t="inlineStr"/>
-      <c r="H64" s="22" t="inlineStr"/>
-      <c r="I64" s="22" t="inlineStr"/>
+      <c r="H64" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I64" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/654878a0-3862-47d1-02aa-550b493fce00/w=365,h=359</t>
+        </is>
+      </c>
       <c r="J64" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-moteur-motorbike/liqui-moly-huile-moteur-motorbike/liqui-moly-motorbike-4t-10w-30-street-1l/</t>
@@ -7069,17 +8108,33 @@
           <t>liqui-moly-motorbike-huile-transmission-75w90-500ml</t>
         </is>
       </c>
-      <c r="C65" s="15" t="inlineStr"/>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>LM1516</t>
+        </is>
+      </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E65" s="16" t="inlineStr"/>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F65" s="16" t="inlineStr"/>
       <c r="G65" s="16" t="inlineStr"/>
-      <c r="H65" s="16" t="inlineStr"/>
-      <c r="I65" s="16" t="inlineStr"/>
+      <c r="H65" s="16" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I65" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/89a51a17-5268-420d-d413-d24a080ffc00/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J65" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-transmission/liqui-moly-motorbike-huile-transmission-75w90-500ml/</t>
@@ -7096,17 +8151,33 @@
           <t>liqui-moly-motorbike-huile-transmission-80w90-150ml</t>
         </is>
       </c>
-      <c r="C66" s="21" t="inlineStr"/>
+      <c r="C66" s="21" t="inlineStr">
+        <is>
+          <t>LM5929</t>
+        </is>
+      </c>
       <c r="D66" s="22" t="inlineStr">
         <is>
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E66" s="22" t="inlineStr"/>
+      <c r="E66" s="22" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
       <c r="F66" s="22" t="inlineStr"/>
       <c r="G66" s="22" t="inlineStr"/>
-      <c r="H66" s="22" t="inlineStr"/>
-      <c r="I66" s="22" t="inlineStr"/>
+      <c r="H66" s="22" t="inlineStr">
+        <is>
+          <t>Votre panier est vide.</t>
+        </is>
+      </c>
+      <c r="I66" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/7dd6e2a6-8d2e-49eb-7ac4-3091b3e35900/w=600,h=600,fit=crop</t>
+        </is>
+      </c>
       <c r="J66" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-transmission/liqui-moly-motorbike-huile-transmission-80w90-150ml/</t>
@@ -7129,11 +8200,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E67" s="16" t="inlineStr"/>
-      <c r="F67" s="16" t="inlineStr"/>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>97.90</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G67" s="16" t="inlineStr"/>
-      <c r="H67" s="16" t="inlineStr"/>
-      <c r="I67" s="16" t="inlineStr"/>
+      <c r="H67" s="16" t="inlineStr">
+        <is>
+          <t>💡 +200% luminosité par rapport aux normes minimales légales</t>
+        </is>
+      </c>
+      <c r="I67" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/6387ff00-bed7-4098-08dd-1915b91f9a00/w=365</t>
+        </is>
+      </c>
       <c r="J67" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huile-transmission/liqui-moly-huile-transmission-10w30-1l/</t>
@@ -7156,11 +8243,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E68" s="22" t="inlineStr"/>
-      <c r="F68" s="22" t="inlineStr"/>
+      <c r="E68" s="22" t="inlineStr">
+        <is>
+          <t>29.90</t>
+        </is>
+      </c>
+      <c r="F68" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G68" s="22" t="inlineStr"/>
-      <c r="H68" s="22" t="inlineStr"/>
-      <c r="I68" s="22" t="inlineStr"/>
+      <c r="H68" s="22" t="inlineStr">
+        <is>
+          <t>💡 Halogène haute performance H9</t>
+        </is>
+      </c>
+      <c r="I68" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/67b526f9-9dee-41fb-fe3e-4e89cc778000/w=600</t>
+        </is>
+      </c>
       <c r="J68" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huiles-pour-fourche/liqui-moly-motorbike-huile-fourche-10w-medium-500ml/</t>
@@ -7183,11 +8286,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E69" s="16" t="inlineStr"/>
-      <c r="F69" s="16" t="inlineStr"/>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>13.99</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G69" s="16" t="inlineStr"/>
-      <c r="H69" s="16" t="inlineStr"/>
-      <c r="I69" s="16" t="inlineStr"/>
+      <c r="H69" s="16" t="inlineStr">
+        <is>
+          <t>💡 4100 lumens avec portée de 238 mètres en route et tout-terrain</t>
+        </is>
+      </c>
+      <c r="I69" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/058940c3-ebfb-4cfd-270a-956dfe43fd00/w=600</t>
+        </is>
+      </c>
       <c r="J69" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huiles-pour-fourche/liqui-moly-motorbike-huile-fourche-5w-light-500ml/</t>
@@ -7210,11 +8329,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E70" s="22" t="inlineStr"/>
-      <c r="F70" s="22" t="inlineStr"/>
+      <c r="E70" s="22" t="inlineStr">
+        <is>
+          <t>16.90</t>
+        </is>
+      </c>
+      <c r="F70" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G70" s="22" t="inlineStr"/>
-      <c r="H70" s="22" t="inlineStr"/>
-      <c r="I70" s="22" t="inlineStr"/>
+      <c r="H70" s="22" t="inlineStr">
+        <is>
+          <t>💡 Feu auxiliaire 6 LED longue portée 190m</t>
+        </is>
+      </c>
+      <c r="I70" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/5ec9712b-a588-4503-d8e5-6c571e100a00/w=600</t>
+        </is>
+      </c>
       <c r="J70" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/huiles-pour-fourche/liqui-moly-motorbike-huile-fourche-15w-heavy-500ml/</t>
@@ -7237,11 +8372,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E71" s="16" t="inlineStr"/>
-      <c r="F71" s="16" t="inlineStr"/>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>199.90</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G71" s="16" t="inlineStr"/>
-      <c r="H71" s="16" t="inlineStr"/>
-      <c r="I71" s="16" t="inlineStr"/>
+      <c r="H71" s="16" t="inlineStr">
+        <is>
+          <t>💡 9 LED performantes, portée 318 mètres.</t>
+        </is>
+      </c>
+      <c r="I71" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/6d4a6511-751b-4cf9-e4e2-a98b98d99c00/w=600</t>
+        </is>
+      </c>
       <c r="J71" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/liqui-moly-nettoyant-pour-chaines-et-freins/</t>
@@ -7264,11 +8415,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E72" s="22" t="inlineStr"/>
-      <c r="F72" s="22" t="inlineStr"/>
+      <c r="E72" s="22" t="inlineStr">
+        <is>
+          <t>199.90</t>
+        </is>
+      </c>
+      <c r="F72" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G72" s="22" t="inlineStr"/>
-      <c r="H72" s="22" t="inlineStr"/>
-      <c r="I72" s="22" t="inlineStr"/>
+      <c r="H72" s="22" t="inlineStr">
+        <is>
+          <t>💡 Luminosité +120% vs norme ECE R112 minimale</t>
+        </is>
+      </c>
+      <c r="I72" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a1dfb9ed-37db-4c74-9498-030b051f1500/w=940</t>
+        </is>
+      </c>
       <c r="J72" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/liqui-moly-pack-entretien-moto/</t>
@@ -7291,11 +8458,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E73" s="16" t="inlineStr"/>
-      <c r="F73" s="16" t="inlineStr"/>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>259.90</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G73" s="16" t="inlineStr"/>
-      <c r="H73" s="16" t="inlineStr"/>
-      <c r="I73" s="16" t="inlineStr"/>
+      <c r="H73" s="16" t="inlineStr">
+        <is>
+          <t>💡 Luminosité +300% vs norme ECE R112 pour visibilité optimale</t>
+        </is>
+      </c>
+      <c r="I73" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/ce72457c-4106-4684-d314-1cebe02b5b00/w=600</t>
+        </is>
+      </c>
       <c r="J73" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/graisse-de-chaine/liqui-moly-motorbike-graisse-de-chaine-blanche-400ml/</t>
@@ -7318,11 +8501,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E74" s="22" t="inlineStr"/>
-      <c r="F74" s="22" t="inlineStr"/>
+      <c r="E74" s="22" t="inlineStr">
+        <is>
+          <t>64.90</t>
+        </is>
+      </c>
+      <c r="F74" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G74" s="22" t="inlineStr"/>
-      <c r="H74" s="22" t="inlineStr"/>
-      <c r="I74" s="22" t="inlineStr"/>
+      <c r="H74" s="22" t="inlineStr">
+        <is>
+          <t>💡 Luminosité standard fiable et stable</t>
+        </is>
+      </c>
+      <c r="I74" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/aa2b894a-0887-4445-0a3c-b40a50e8f700/w=1000</t>
+        </is>
+      </c>
       <c r="J74" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/accessoires-moto/pack-entretien-chaine-premium-liqui-moly/</t>
@@ -7345,11 +8544,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E75" s="16" t="inlineStr"/>
-      <c r="F75" s="16" t="inlineStr"/>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>299.90</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G75" s="16" t="inlineStr"/>
-      <c r="H75" s="16" t="inlineStr"/>
-      <c r="I75" s="16" t="inlineStr"/>
+      <c r="H75" s="16" t="inlineStr">
+        <is>
+          <t>💡 LED blanc froid 6000K pour phares modernes</t>
+        </is>
+      </c>
+      <c r="I75" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a199f886-97df-4048-a817-50ac25586500/w=600</t>
+        </is>
+      </c>
       <c r="J75" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/graisse-de-chaine/liqui-moly-motorbike-graisse-de-chaine-250ml/</t>
@@ -7372,11 +8587,27 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E76" s="22" t="inlineStr"/>
-      <c r="F76" s="22" t="inlineStr"/>
+      <c r="E76" s="22" t="inlineStr">
+        <is>
+          <t>189.90</t>
+        </is>
+      </c>
+      <c r="F76" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G76" s="22" t="inlineStr"/>
-      <c r="H76" s="22" t="inlineStr"/>
-      <c r="I76" s="22" t="inlineStr"/>
+      <c r="H76" s="22" t="inlineStr">
+        <is>
+          <t>💡 14 LED haute performance, portée 36 mètres.</t>
+        </is>
+      </c>
+      <c r="I76" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/69ae8e58-82f2-457b-b564-4f2e8c7fe600/w=600</t>
+        </is>
+      </c>
       <c r="J76" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/liqui-moly-nettoyant-radiateur/</t>
@@ -7399,11 +8630,23 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E77" s="16" t="inlineStr"/>
-      <c r="F77" s="16" t="inlineStr"/>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>14.90</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G77" s="16" t="inlineStr"/>
       <c r="H77" s="16" t="inlineStr"/>
-      <c r="I77" s="16" t="inlineStr"/>
+      <c r="I77" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a8cc3a63-1857-45bd-2e66-e999045f4a00/w=600</t>
+        </is>
+      </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/additifs-moto/additif-huile/liqui-moly-engine-flush-shooter/</t>
@@ -7426,11 +8669,23 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E78" s="22" t="inlineStr"/>
-      <c r="F78" s="22" t="inlineStr"/>
+      <c r="E78" s="22" t="inlineStr">
+        <is>
+          <t>47.90</t>
+        </is>
+      </c>
+      <c r="F78" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G78" s="22" t="inlineStr"/>
       <c r="H78" s="22" t="inlineStr"/>
-      <c r="I78" s="22" t="inlineStr"/>
+      <c r="I78" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/43146794-b896-429f-0c0b-7e0342c16000/w=600</t>
+        </is>
+      </c>
       <c r="J78" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/motorbike/entretien-moto/liqui-moly-nettoyant-moto/</t>
@@ -7453,11 +8708,23 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E79" s="16" t="inlineStr"/>
-      <c r="F79" s="16" t="inlineStr"/>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>29.90</t>
+        </is>
+      </c>
+      <c r="F79" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G79" s="16" t="inlineStr"/>
       <c r="H79" s="16" t="inlineStr"/>
-      <c r="I79" s="16" t="inlineStr"/>
+      <c r="I79" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/bc24faeb-febe-4f3b-848e-725df0c0fa00/w=1772</t>
+        </is>
+      </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/nettoyant-injection/liqui-moly-nettoyant-pour-systemes-dinjection-essence-300ml/</t>
@@ -7480,11 +8747,23 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E80" s="22" t="inlineStr"/>
-      <c r="F80" s="22" t="inlineStr"/>
+      <c r="E80" s="22" t="inlineStr">
+        <is>
+          <t>59.90</t>
+        </is>
+      </c>
+      <c r="F80" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G80" s="22" t="inlineStr"/>
       <c r="H80" s="22" t="inlineStr"/>
-      <c r="I80" s="22" t="inlineStr"/>
+      <c r="I80" s="23" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/74464be7-5b1b-478f-9f88-153892867500/w=600</t>
+        </is>
+      </c>
       <c r="J80" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/nettoyant-injection/liqui-moly-nettoyant-pour-systeme-diesel-pro-line-500ml/</t>
@@ -7507,11 +8786,23 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E81" s="16" t="inlineStr"/>
-      <c r="F81" s="16" t="inlineStr"/>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>44.90</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G81" s="16" t="inlineStr"/>
       <c r="H81" s="16" t="inlineStr"/>
-      <c r="I81" s="16" t="inlineStr"/>
+      <c r="I81" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a92673cd-6330-419e-70a8-8840fe621e00/w=600</t>
+        </is>
+      </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/nettoyant-injection/liqui-moly-pro-line-systeme-nettoyant-pour-essence/</t>
@@ -7534,11 +8825,23 @@
           <t>Liqui Moly</t>
         </is>
       </c>
-      <c r="E82" s="22" t="inlineStr"/>
-      <c r="F82" s="22" t="inlineStr"/>
+      <c r="E82" s="22" t="inlineStr">
+        <is>
+          <t>24.90</t>
+        </is>
+      </c>
+      <c r="F82" s="22" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G82" s="22" t="inlineStr"/>
       <c r="H82" s="22" t="inlineStr"/>
-      <c r="I82" s="22" t="inlineStr"/>
+      <c r="I82" s="23" t="inlineStr">
+        <is>
+          <t>https://tomobile.store/wp-content/uploads/2026/01/6a790eed1d8f2384fc9a399eac0ac08b8bc457a6_1515_Marderspray_200ml_8c59-1.jpg]</t>
+        </is>
+      </c>
       <c r="J82" s="23" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/produits-dentretien/liqui-moly-anti-rongeurs/</t>
@@ -7578,71 +8881,136 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId156"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8416,11 +9784,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E18" s="25" t="inlineStr"/>
-      <c r="F18" s="25" t="inlineStr"/>
+      <c r="E18" s="25" t="inlineStr">
+        <is>
+          <t>1,084.90</t>
+        </is>
+      </c>
+      <c r="F18" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G18" s="25" t="inlineStr"/>
-      <c r="H18" s="25" t="inlineStr"/>
-      <c r="I18" s="25" t="inlineStr"/>
+      <c r="H18" s="25" t="inlineStr">
+        <is>
+          <t>💡 12 LED haute performance, portée 300 mètres.</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/4d54d113-8310-4f86-3c0d-d3257a00da00/w=900</t>
+        </is>
+      </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/feux-auxiliaire/osram-phare-ledriving-mx180-cb/</t>
@@ -8443,11 +9827,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr"/>
-      <c r="F19" s="16" t="inlineStr"/>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>29.90</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G19" s="16" t="inlineStr"/>
-      <c r="H19" s="16" t="inlineStr"/>
-      <c r="I19" s="16" t="inlineStr"/>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>💡 Blanc bleuté intense jusqu’à 4200K aspect xénon premium</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/488a9fdb-cb24-4089-38f6-1d34fdef5e00/w=900</t>
+        </is>
+      </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h7/osram-h7-cool-blue-intense-aspect-xenon/</t>
@@ -8470,11 +9870,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E20" s="25" t="inlineStr"/>
-      <c r="F20" s="25" t="inlineStr"/>
+      <c r="E20" s="25" t="inlineStr">
+        <is>
+          <t>9.90</t>
+        </is>
+      </c>
+      <c r="F20" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G20" s="25" t="inlineStr"/>
-      <c r="H20" s="25" t="inlineStr"/>
-      <c r="I20" s="25" t="inlineStr"/>
+      <c r="H20" s="25" t="inlineStr">
+        <is>
+          <t>💡 Ampoule halogène H7 55W 12V — culot PX26d, catégorie ECE H7</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/be5b1277-9dfa-46c6-3194-bae2fa3fdd00/w=900</t>
+        </is>
+      </c>
       <c r="J20" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h7/osram-original-line-h7-55w-12v/</t>
@@ -8497,11 +9913,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr"/>
-      <c r="F21" s="16" t="inlineStr"/>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>42.90</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G21" s="16" t="inlineStr"/>
-      <c r="H21" s="16" t="inlineStr"/>
-      <c r="I21" s="16" t="inlineStr"/>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>💡 100% plus de lumière que la norme légale minimum</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/e0bea2a1-affc-4574-8c28-0dc8f21a1f00/w=900</t>
+        </is>
+      </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h7/osram-night-breaker-silver-100-h7/</t>
@@ -8524,11 +9956,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E22" s="25" t="inlineStr"/>
-      <c r="F22" s="25" t="inlineStr"/>
+      <c r="E22" s="25" t="inlineStr">
+        <is>
+          <t>64.90</t>
+        </is>
+      </c>
+      <c r="F22" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G22" s="25" t="inlineStr"/>
-      <c r="H22" s="25" t="inlineStr"/>
-      <c r="I22" s="25" t="inlineStr"/>
+      <c r="H22" s="25" t="inlineStr">
+        <is>
+          <t>💡 Blanc froid 6000K pour visibilité maximale et look premium</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/59328f16-dabd-4eb6-4d4f-226217e4e800/w=900</t>
+        </is>
+      </c>
       <c r="J22" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h7/osram-ultra-life-h7/</t>
@@ -8551,11 +9999,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr"/>
-      <c r="F23" s="16" t="inlineStr"/>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>9.90</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G23" s="16" t="inlineStr"/>
-      <c r="H23" s="16" t="inlineStr"/>
-      <c r="I23" s="16" t="inlineStr"/>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>💡 280 lumens – visibilité optimale</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/99660ee4-97e0-4a39-113a-3eca251ef500/w=728</t>
+        </is>
+      </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h7/osram-night-breaker-200-h7/</t>
@@ -8578,11 +10042,23 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E24" s="25" t="inlineStr"/>
-      <c r="F24" s="25" t="inlineStr"/>
+      <c r="E24" s="25" t="inlineStr">
+        <is>
+          <t>59.90</t>
+        </is>
+      </c>
+      <c r="F24" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G24" s="25" t="inlineStr"/>
       <c r="H24" s="25" t="inlineStr"/>
-      <c r="I24" s="25" t="inlineStr"/>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a96a3cb8-db57-4a23-c81c-c151351d9d00/w=900</t>
+        </is>
+      </c>
       <c r="J24" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h9/osram-h9/</t>
@@ -8605,11 +10081,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr"/>
-      <c r="F25" s="16" t="inlineStr"/>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>13.99</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G25" s="16" t="inlineStr"/>
-      <c r="H25" s="16" t="inlineStr"/>
-      <c r="I25" s="16" t="inlineStr"/>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>💡 4100 lumens avec portée de 238 mètres en route et tout-terrain</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/d108e8ce-b7bf-4864-4936-475bae557a00/w=900</t>
+        </is>
+      </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/feux-auxiliaire/osram-barre-led-vx500-cb/</t>
@@ -8632,11 +10124,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E26" s="25" t="inlineStr"/>
-      <c r="F26" s="25" t="inlineStr"/>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>16.90</t>
+        </is>
+      </c>
+      <c r="F26" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G26" s="25" t="inlineStr"/>
-      <c r="H26" s="25" t="inlineStr"/>
-      <c r="I26" s="25" t="inlineStr"/>
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>💡 Feu auxiliaire 6 LED longue portée 190m</t>
+        </is>
+      </c>
+      <c r="I26" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/578d86b1-0d8e-482c-3110-5508b9aeec00/w=900</t>
+        </is>
+      </c>
       <c r="J26" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/feux-auxiliaire/osram-barre-led-sx180-sp/</t>
@@ -8659,11 +10167,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr"/>
-      <c r="F27" s="16" t="inlineStr"/>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>199.90</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G27" s="16" t="inlineStr"/>
-      <c r="H27" s="16" t="inlineStr"/>
-      <c r="I27" s="16" t="inlineStr"/>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>💡 9 LED performantes, portée 318 mètres.</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/10ebd953-3112-45de-54ca-f6b76b591200/w=900</t>
+        </is>
+      </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/feux-auxiliaire/osram-barre-led-vx250-sp/</t>
@@ -8686,11 +10210,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E28" s="25" t="inlineStr"/>
-      <c r="F28" s="25" t="inlineStr"/>
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>199.90</t>
+        </is>
+      </c>
+      <c r="F28" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G28" s="25" t="inlineStr"/>
-      <c r="H28" s="25" t="inlineStr"/>
-      <c r="I28" s="25" t="inlineStr"/>
+      <c r="H28" s="25" t="inlineStr">
+        <is>
+          <t>💡 Luminosité +120% vs norme ECE R112 minimale</t>
+        </is>
+      </c>
+      <c r="I28" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/2afd1bea-b6ab-46a8-afac-ef2ef32f4400/w=1080</t>
+        </is>
+      </c>
       <c r="J28" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h1/osram-ledriving-spk-h1/</t>
@@ -8713,11 +10253,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr"/>
-      <c r="F29" s="16" t="inlineStr"/>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t>259.90</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G29" s="16" t="inlineStr"/>
-      <c r="H29" s="16" t="inlineStr"/>
-      <c r="I29" s="16" t="inlineStr"/>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>💡 Luminosité +300% vs norme ECE R112 pour visibilité optimale</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/c6d1f2ae-776e-4a96-66c7-24131334c400/w=1080</t>
+        </is>
+      </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/h1/osram-ledriving-hl-bright-h1/</t>
@@ -8740,11 +10296,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E30" s="25" t="inlineStr"/>
-      <c r="F30" s="25" t="inlineStr"/>
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>64.90</t>
+        </is>
+      </c>
+      <c r="F30" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G30" s="25" t="inlineStr"/>
-      <c r="H30" s="25" t="inlineStr"/>
-      <c r="I30" s="25" t="inlineStr"/>
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>💡 Luminosité standard fiable et stable</t>
+        </is>
+      </c>
+      <c r="I30" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/b02a1d2c-43c8-40c1-fa8b-25e77c1c1d00/w=900</t>
+        </is>
+      </c>
       <c r="J30" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/led/osram-h15/</t>
@@ -8767,11 +10339,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr"/>
-      <c r="F31" s="16" t="inlineStr"/>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>299.90</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G31" s="16" t="inlineStr"/>
-      <c r="H31" s="16" t="inlineStr"/>
-      <c r="I31" s="16" t="inlineStr"/>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>💡 LED blanc froid 6000K pour phares modernes</t>
+        </is>
+      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/abec0804-b0b9-402c-3839-42f9449e5e00/w=900</t>
+        </is>
+      </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/led/osram-kit-led-h7-hl-gen-2/</t>
@@ -8794,11 +10382,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E32" s="25" t="inlineStr"/>
-      <c r="F32" s="25" t="inlineStr"/>
+      <c r="E32" s="25" t="inlineStr">
+        <is>
+          <t>189.90</t>
+        </is>
+      </c>
+      <c r="F32" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G32" s="25" t="inlineStr"/>
-      <c r="H32" s="25" t="inlineStr"/>
-      <c r="I32" s="25" t="inlineStr"/>
+      <c r="H32" s="25" t="inlineStr">
+        <is>
+          <t>💡 14 LED haute performance, portée 36 mètres.</t>
+        </is>
+      </c>
+      <c r="I32" s="26" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/c6c694be-6be0-4fc5-cce2-59ed40412900/w=900</t>
+        </is>
+      </c>
       <c r="J32" s="26" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/feux-auxiliaire/osram-reversing-led-fx120r-wd/</t>
@@ -8821,11 +10425,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr"/>
-      <c r="F33" s="16" t="inlineStr"/>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>64.90</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G33" s="16" t="inlineStr"/>
-      <c r="H33" s="16" t="inlineStr"/>
-      <c r="I33" s="16" t="inlineStr"/>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>💡 13 LED haute intensité, portée 36 mètres.</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/5dc170da-d7b4-4f40-fda1-ad46451b0e00/w=900</t>
+        </is>
+      </c>
       <c r="J33" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/feux-auxiliaire/osram-reversing-fx120s-wd/</t>
@@ -8848,10 +10468,22 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E34" s="25" t="inlineStr"/>
-      <c r="F34" s="25" t="inlineStr"/>
+      <c r="E34" s="25" t="inlineStr">
+        <is>
+          <t>64.90</t>
+        </is>
+      </c>
+      <c r="F34" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G34" s="25" t="inlineStr"/>
-      <c r="H34" s="25" t="inlineStr"/>
+      <c r="H34" s="25" t="inlineStr">
+        <is>
+          <t>💡 Blanc froid 6000K pour visibilité maximale et look premium</t>
+        </is>
+      </c>
       <c r="I34" s="25" t="inlineStr"/>
       <c r="J34" s="26" t="inlineStr">
         <is>
@@ -8875,11 +10507,27 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr"/>
-      <c r="F35" s="16" t="inlineStr"/>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>9.90</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G35" s="16" t="inlineStr"/>
-      <c r="H35" s="16" t="inlineStr"/>
-      <c r="I35" s="16" t="inlineStr"/>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>💡 280 lumens – visibilité optimale</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
+        <is>
+          <t>https://imagedelivery.net/q8VWDJbIll_I_5B7drMkig/a0cc3e70-e778-4528-c38f-c98a1629d000/w=900</t>
+        </is>
+      </c>
       <c r="J35" s="17" t="inlineStr">
         <is>
           <t>https://tomobile.store/shop/eclairage-automobile/signalisation/osram-lampe-wx3x16d-orange/</t>
@@ -8902,8 +10550,16 @@
           <t>Osram</t>
         </is>
       </c>
-      <c r="E36" s="25" t="inlineStr"/>
-      <c r="F36" s="25" t="inlineStr"/>
+      <c r="E36" s="25" t="inlineStr">
+        <is>
+          <t>59.90</t>
+        </is>
+      </c>
+      <c r="F36" s="25" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
       <c r="G36" s="25" t="inlineStr"/>
       <c r="H36" s="25" t="inlineStr"/>
       <c r="I36" s="25" t="inlineStr"/>
@@ -8946,25 +10602,42 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>